<commit_message>
docs: record founder answers Q-F01 to Q-F03, Q-F05, Q-F06
Indian company, ₹5,000-10,000 monthly budget, January 2027 beta,
5 free commercial songs per month, 30-50 developer hours a week.
Adds DEC-022 to DEC-026, updates assumptions, budget plan and sprint capacity.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KC7q2XdCVxuwsART7HEcsQ
</commit_message>
<xml_diff>
--- a/docs/13-business/financial-model.xlsx
+++ b/docs/13-business/financial-model.xlsx
@@ -805,7 +805,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -814,12 +814,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>[A]</t>
+          <t>[SS]</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Q-F02 default ₹0</t>
+          <t>DEC-023: ₹5,000 to ₹10,000; floor used</t>
         </is>
       </c>
     </row>
@@ -3325,12 +3325,12 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Pre-funding monthly budget (Q-F02)</t>
+          <t>Pre-funding monthly budget (DEC-023)</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>₹0</t>
+          <t>₹5,000</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
@@ -3338,11 +3338,7 @@
           <t>₹10,000</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>₹50,000</t>
-        </is>
-      </c>
+      <c r="D3" s="1" t="inlineStr"/>
       <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
@@ -3356,14 +3352,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="C4" t="n">
         <v>0.6</v>
       </c>
-      <c r="D4" t="n">
-        <v>0.55</v>
-      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>Largest variable cost; credits first</t>
@@ -3377,14 +3370,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="C5" t="n">
         <v>0.1</v>
       </c>
-      <c r="D5" t="n">
-        <v>0.05</v>
-      </c>
       <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
@@ -3394,14 +3384,11 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="C6" t="n">
         <v>0.15</v>
       </c>
-      <c r="D6" t="n">
-        <v>0.15</v>
-      </c>
       <c r="E6" t="inlineStr">
         <is>
           <t>Evidence for investors</t>
@@ -3415,14 +3402,11 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="C7" t="n">
         <v>0.15</v>
       </c>
-      <c r="D7" t="n">
-        <v>0.15</v>
-      </c>
       <c r="E7" t="inlineStr">
         <is>
           <t>Needs quotes</t>
@@ -3441,12 +3425,9 @@
       <c r="C8" t="n">
         <v>0</v>
       </c>
-      <c r="D8" t="n">
-        <v>0.1</v>
-      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Or pay one-off from savings before paid launch</t>
+          <t>Pay one-off from savings before paid launch</t>
         </is>
       </c>
     </row>
@@ -3462,10 +3443,6 @@
       </c>
       <c r="C9">
         <f>SUM(C4:C8)</f>
-        <v/>
-      </c>
-      <c r="D9">
-        <f>SUM(D4:D8)</f>
         <v/>
       </c>
     </row>

</xml_diff>